<commit_message>
upload aula 6 e grupos
</commit_message>
<xml_diff>
--- a/SEMINÁRIO/GRUPOS_SEMINÁRIO.xlsx
+++ b/SEMINÁRIO/GRUPOS_SEMINÁRIO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertvidigal/Documents/2026-2_FPP/2026-2_FPP_Online/SEMINÁRIO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59399481-7459-214F-87D5-251AE0958DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7209787C-E198-9F43-AD4F-E9DBD5BAFE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{F4198FB7-85B9-2942-BFCC-3FF6707350B2}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="FPP2026.2" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FPP2026.2'!$A$1:$C$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FPP2026.2'!$A$1:$C$62</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>NOME</t>
   </si>
@@ -411,13 +411,19 @@
   </si>
   <si>
     <t>GRUPO DO SEMINÁRIO</t>
+  </si>
+  <si>
+    <t>RENAN ALEXANDER SIQUEIRA</t>
+  </si>
+  <si>
+    <t>ras.alexander@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -431,6 +437,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -453,11 +465,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1B06DF2-641D-8643-983E-04031EBF8DDA}">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.1640625" bestFit="1" customWidth="1"/>
@@ -1358,88 +1371,88 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53" t="s">
-        <v>113</v>
+      <c r="A53" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="C53">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C54">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C55">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C56">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C57">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C58">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C59">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C60">
         <v>6</v>
@@ -1447,17 +1460,28 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>60</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B62" t="s">
         <v>121</v>
       </c>
-      <c r="C61">
+      <c r="C62">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C61" xr:uid="{B1B06DF2-641D-8643-983E-04031EBF8DDA}"/>
+  <autoFilter ref="A1:C62" xr:uid="{B1B06DF2-641D-8643-983E-04031EBF8DDA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
upload Aula 7 e 8
</commit_message>
<xml_diff>
--- a/SEMINÁRIO/GRUPOS_SEMINÁRIO.xlsx
+++ b/SEMINÁRIO/GRUPOS_SEMINÁRIO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertvidigal/Documents/2026-2_FPP/2026-2_FPP_Online/SEMINÁRIO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7209787C-E198-9F43-AD4F-E9DBD5BAFE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2555294-0011-2144-B0AD-623EBE26F46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{F4198FB7-85B9-2942-BFCC-3FF6707350B2}"/>
   </bookViews>
@@ -957,6 +957,9 @@
       <c r="B14" t="s">
         <v>74</v>
       </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">

</xml_diff>